<commit_message>
Add README and docs
</commit_message>
<xml_diff>
--- a/OpenBloom_Project_Tracker.xlsx
+++ b/OpenBloom_Project_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Open_bloom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A941817A-1E17-4A8C-9371-E51F6BD7B6D6}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8120000_{FCCA252E-93C3-444A-A3FE-117A65ADE641}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9216" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9216" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>

</xml_diff>